<commit_message>
Update TSLA model and portfolio
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/companies/TSLA.xlsx
+++ b/companies/TSLA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\models\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dillonwalton/Desktop/business/models/companies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8240D41D-D31A-4D07-94CF-69BC3D7A3A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3035A6D-BF85-7B44-815A-FA98245DF29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{969D4ED5-6A32-DE48-841A-E0A03F4B02B5}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" xr2:uid="{969D4ED5-6A32-DE48-841A-E0A03F4B02B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -518,8 +518,45 @@
 </comments>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="180">
   <si>
     <t>Revenue</t>
   </si>
@@ -1056,6 +1093,9 @@
   </si>
   <si>
     <t>10-K</t>
+  </si>
+  <si>
+    <t>Ticker</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1217,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1194,6 +1234,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1320,6 +1362,447 @@
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Dillon Walton" id="{72341B3D-64ED-DE40-92E1-1286D6A616CD}" userId="S::dillon.walton@apexcleanenergy.com::d6a318a4-b905-4bee-a20f-e7b3b62104df" providerId="AD"/>
 </personList>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+  <types>
+    <type name="_linkedentity">
+      <keyFlags>
+        <key name="%cvi">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+          <flag name="ExcludeFromCalcComparison" value="1"/>
+        </key>
+      </keyFlags>
+    </type>
+    <type name="_linkedentitycore">
+      <keyFlags>
+        <key name="%EntityServiceId">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%EntitySubDomainId">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%EntityCulture">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%EntityId">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%IsRefreshable">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+          <flag name="ExcludeFromCalcComparison" value="1"/>
+        </key>
+        <key name="%ProviderInfo">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%DataProviderExternalLinkLogo">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%DataProviderExternalLink">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+        </key>
+        <key name="%OutdatedReason">
+          <flag name="ShowInCardView" value="0"/>
+          <flag name="ShowInDotNotation" value="0"/>
+          <flag name="ShowInAutoComplete" value="0"/>
+          <flag name="ExcludeFromCalcComparison" value="1"/>
+        </key>
+      </keyFlags>
+    </type>
+  </types>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
+  <rv s="0">
+    <v>https://www.bing.com/financeapi/forcetrigger?t=a24kar&amp;q=XNAS%3aTSLA&amp;form=skydnc</v>
+    <v>Learn more on Bing</v>
+  </rv>
+  <rv s="1">
+    <v>0</v>
+    <v>TESLA, INC. (XNAS:TSLA)</v>
+    <v>2</v>
+    <v>3</v>
+    <v>Finance</v>
+    <v>4</v>
+    <v>en-US</v>
+    <v>a24kar</v>
+    <v>268435456</v>
+    <v>1</v>
+    <v>Powered by Refinitiv</v>
+    <v>498.83</v>
+    <v>297.38</v>
+    <v>1.9121999999999999</v>
+    <v>1.22</v>
+    <v>3.2200000000000002E-3</v>
+    <v>1.3899999999999999E-2</v>
+    <v>3.6570000000000004E-5</v>
+    <v>USD</v>
+    <v>Tesla, Inc. designs, develops, manufactures, sells and leases high-performance fully electric vehicles and energy generation and storage systems, and offers services related to its products. Its segments include automotive, and energy generation and storage. The automotive segment includes the design, development, manufacturing, sales and leasing of high-performance fully electric vehicles, and sales of automotive regulatory credits. It also includes sales of used vehicles, non-warranty maintenance services and collisions, part sales, paid supercharging, insurance services revenue and retail merchandise sales. The energy generation and storage segment include the design, manufacture, installation, sales and leasing of solar energy generation and energy storage products and related services and sales of solar energy systems incentives. Its consumer vehicles include the Model 3, Y, S, X and Cybertruck. Its lithium-ion battery energy storage products include Powerwall and Megapack.</v>
+    <v>134785</v>
+    <v>Nasdaq Stock Market</v>
+    <v>XNAS</v>
+    <v>XNAS</v>
+    <v>1 Tesla Road, AUSTIN, TX, 78725 US</v>
+    <v>386.7</v>
+    <v>Automobiles &amp; Auto Parts</v>
+    <v>Stock</v>
+    <v>46288.999961863279</v>
+    <v>0</v>
+    <v>377.57499999999999</v>
+    <v>1501301805640</v>
+    <v>TESLA, INC.</v>
+    <v>TESLA, INC.</v>
+    <v>380.1</v>
+    <v>380.42430000000002</v>
+    <v>378.9</v>
+    <v>380.12</v>
+    <v>380.13389999999998</v>
+    <v>3949547000</v>
+    <v>TSLA</v>
+    <v>TESLA, INC. (XNAS:TSLA)</v>
+    <v>33522492</v>
+    <v>38800703</v>
+    <v>2024</v>
+  </rv>
+  <rv s="2">
+    <v>1</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
+  <s t="_hyperlink">
+    <k n="Address" t="s"/>
+    <k n="Text" t="s"/>
+  </s>
+  <s t="_linkedentitycore">
+    <k n="_Display" t="spb"/>
+    <k n="_DisplayString" t="s"/>
+    <k n="_Flags" t="spb"/>
+    <k n="_Format" t="spb"/>
+    <k n="_Icon" t="s"/>
+    <k n="_SubLabel" t="spb"/>
+    <k n="%EntityCulture" t="s"/>
+    <k n="%EntityId" t="s"/>
+    <k n="%EntityServiceId"/>
+    <k n="%IsRefreshable" t="b"/>
+    <k n="%ProviderInfo" t="s"/>
+    <k n="52 week high"/>
+    <k n="52 week low"/>
+    <k n="Beta"/>
+    <k n="Change"/>
+    <k n="Change (%)"/>
+    <k n="Change (Extended hours)"/>
+    <k n="Change % (Extended hours)"/>
+    <k n="Currency" t="s"/>
+    <k n="Description" t="s"/>
+    <k n="Employees"/>
+    <k n="Exchange" t="s"/>
+    <k n="Exchange abbreviation" t="s"/>
+    <k n="ExchangeID" t="s"/>
+    <k n="Headquarters" t="s"/>
+    <k n="High"/>
+    <k n="Industry" t="s"/>
+    <k n="Instrument type" t="s"/>
+    <k n="Last trade time"/>
+    <k n="LearnMoreOnLink" t="r"/>
+    <k n="Low"/>
+    <k n="Market cap"/>
+    <k n="Name" t="s"/>
+    <k n="Official name" t="s"/>
+    <k n="Open"/>
+    <k n="P/E"/>
+    <k n="Previous close"/>
+    <k n="Price"/>
+    <k n="Price (Extended hours)"/>
+    <k n="Shares outstanding"/>
+    <k n="Ticker symbol" t="s"/>
+    <k n="UniqueName" t="s"/>
+    <k n="Volume"/>
+    <k n="Volume average"/>
+    <k n="Year incorporated"/>
+  </s>
+  <s t="_linkedentity">
+    <k n="%cvi" t="r"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
+<supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
+  <spbArrays count="1">
+    <a count="45">
+      <v t="s">%EntityServiceId</v>
+      <v t="s">_Format</v>
+      <v t="s">%IsRefreshable</v>
+      <v t="s">%EntityCulture</v>
+      <v t="s">%EntityId</v>
+      <v t="s">_Icon</v>
+      <v t="s">_Display</v>
+      <v t="s">Name</v>
+      <v t="s">_SubLabel</v>
+      <v t="s">Price</v>
+      <v t="s">Price (Extended hours)</v>
+      <v t="s">Exchange</v>
+      <v t="s">Official name</v>
+      <v t="s">Last trade time</v>
+      <v t="s">Ticker symbol</v>
+      <v t="s">Exchange abbreviation</v>
+      <v t="s">Change</v>
+      <v t="s">Change (Extended hours)</v>
+      <v t="s">Change (%)</v>
+      <v t="s">Change % (Extended hours)</v>
+      <v t="s">Currency</v>
+      <v t="s">Previous close</v>
+      <v t="s">Open</v>
+      <v t="s">High</v>
+      <v t="s">Low</v>
+      <v t="s">52 week high</v>
+      <v t="s">52 week low</v>
+      <v t="s">Volume</v>
+      <v t="s">Volume average</v>
+      <v t="s">Market cap</v>
+      <v t="s">Beta</v>
+      <v t="s">P/E</v>
+      <v t="s">Shares outstanding</v>
+      <v t="s">Description</v>
+      <v t="s">Employees</v>
+      <v t="s">Headquarters</v>
+      <v t="s">Industry</v>
+      <v t="s">Instrument type</v>
+      <v t="s">Year incorporated</v>
+      <v t="s">_Flags</v>
+      <v t="s">UniqueName</v>
+      <v t="s">_DisplayString</v>
+      <v t="s">LearnMoreOnLink</v>
+      <v t="s">ExchangeID</v>
+      <v t="s">%ProviderInfo</v>
+    </a>
+  </spbArrays>
+  <spbData count="5">
+    <spb s="0">
+      <v>0</v>
+      <v>Name</v>
+      <v>LearnMoreOnLink</v>
+    </spb>
+    <spb s="1">
+      <v>0</v>
+      <v>0</v>
+      <v>0</v>
+    </spb>
+    <spb s="2">
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
+    </spb>
+    <spb s="3">
+      <v>1</v>
+      <v>2</v>
+      <v>2</v>
+      <v>1</v>
+      <v>3</v>
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
+      <v>4</v>
+      <v>4</v>
+      <v>5</v>
+      <v>6</v>
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
+      <v>4</v>
+      <v>7</v>
+      <v>8</v>
+      <v>9</v>
+      <v>4</v>
+      <v>1</v>
+      <v>1</v>
+      <v>5</v>
+    </spb>
+    <spb s="4">
+      <v>at close</v>
+      <v>from previous close</v>
+      <v>from previous close</v>
+      <v>Source: Nasdaq</v>
+      <v>GMT</v>
+      <v>Delayed 15 minutes</v>
+      <v>from close</v>
+      <v>from close</v>
+    </spb>
+  </spbData>
+</supportingPropertyBags>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybagstructure.xml><?xml version="1.0" encoding="utf-8"?>
+<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="5">
+  <s>
+    <k n="^Order" t="spba"/>
+    <k n="TitleProperty" t="s"/>
+    <k n="SubTitleProperty" t="s"/>
+  </s>
+  <s>
+    <k n="ShowInCardView" t="b"/>
+    <k n="ShowInDotNotation" t="b"/>
+    <k n="ShowInAutoComplete" t="b"/>
+  </s>
+  <s>
+    <k n="ExchangeID" t="spb"/>
+    <k n="UniqueName" t="spb"/>
+    <k n="`%ProviderInfo" t="spb"/>
+    <k n="LearnMoreOnLink" t="spb"/>
+  </s>
+  <s>
+    <k n="Low" t="i"/>
+    <k n="P/E" t="i"/>
+    <k n="Beta" t="i"/>
+    <k n="High" t="i"/>
+    <k n="Name" t="i"/>
+    <k n="Open" t="i"/>
+    <k n="Price" t="i"/>
+    <k n="Change" t="i"/>
+    <k n="Volume" t="i"/>
+    <k n="Employees" t="i"/>
+    <k n="Change (%)" t="i"/>
+    <k n="Market cap" t="i"/>
+    <k n="52 week low" t="i"/>
+    <k n="52 week high" t="i"/>
+    <k n="Previous close" t="i"/>
+    <k n="Volume average" t="i"/>
+    <k n="Last trade time" t="i"/>
+    <k n="Year incorporated" t="i"/>
+    <k n="`%EntityServiceId" t="i"/>
+    <k n="Shares outstanding" t="i"/>
+    <k n="Price (Extended hours)" t="i"/>
+    <k n="Change (Extended hours)" t="i"/>
+    <k n="Change % (Extended hours)" t="i"/>
+  </s>
+  <s>
+    <k n="Price" t="s"/>
+    <k n="Change" t="s"/>
+    <k n="Change (%)" t="s"/>
+    <k n="ExchangeID" t="s"/>
+    <k n="Last trade time" t="s"/>
+    <k n="Price (Extended hours)" t="s"/>
+    <k n="Change (Extended hours)" t="s"/>
+    <k n="Change % (Extended hours)" t="s"/>
+  </s>
+</spbStructures>
+</file>
+
+<file path=xl/richData/richStyles.xml><?xml version="1.0" encoding="utf-8"?>
+<richStyleSheet xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <dxfs count="7">
+    <x:dxf>
+      <x:numFmt numFmtId="2" formatCode="0.00"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="0" formatCode="General"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="27" formatCode="m/d/yy\ h:mm"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="14" formatCode="0.00%"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="3" formatCode="#,##0"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </x:dxf>
+    <x:dxf>
+      <x:numFmt numFmtId="1" formatCode="0"/>
+    </x:dxf>
+  </dxfs>
+  <richProperties>
+    <rPr n="NumberFormat" t="s"/>
+    <rPr n="IsTitleField" t="b"/>
+  </richProperties>
+  <richStyles>
+    <rSty dxfid="1">
+      <rpv i="0">_([$$-en-US]* #,##0.00_);_([$$-en-US]* (#,##0.00);_([$$-en-US]* "-"??_);_(@_)</rpv>
+    </rSty>
+    <rSty dxfid="5">
+      <rpv i="0">#,##0.00</rpv>
+    </rSty>
+    <rSty>
+      <rpv i="1">1</rpv>
+    </rSty>
+    <rSty dxfid="4">
+      <rpv i="0">#,##0</rpv>
+    </rSty>
+    <rSty dxfid="3"/>
+    <rSty dxfid="1">
+      <rpv i="0">_([$$-en-US]* #,##0_);_([$$-en-US]* (#,##0);_([$$-en-US]* "-"_);_(@_)</rpv>
+    </rSty>
+    <rSty dxfid="2"/>
+    <rSty dxfid="6">
+      <rpv i="0">0</rpv>
+    </rSty>
+    <rSty dxfid="0">
+      <rpv i="0">0.00</rpv>
+    </rSty>
+  </richStyles>
+</richStyleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1748,14 +2231,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA9BD9ED-2B2C-2544-8EDE-5AC0250957CF}">
-  <dimension ref="C4:L34"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="C3:O34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="K3" t="s">
+        <v>179</v>
+      </c>
+      <c r="L3" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="4" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C4" t="s">
         <v>116</v>
       </c>
@@ -1765,11 +2256,24 @@
       <c r="K4" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="1">
-        <v>348.75</v>
-      </c>
-    </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="16" cm="1">
+        <f t="array" aca="1" ref="L4" ca="1">_FV(L3,"Price")</f>
+        <v>380.12</v>
+      </c>
+      <c r="M4" s="16" cm="1">
+        <f t="array" aca="1" ref="M4" ca="1">_FV(L3,"Beta")</f>
+        <v>1.9121999999999999</v>
+      </c>
+      <c r="N4" t="str" cm="1">
+        <f t="array" aca="1" ref="N4" ca="1">_FV(L3,"Industry")</f>
+        <v>Automobiles &amp; Auto Parts</v>
+      </c>
+      <c r="O4" s="17" cm="1">
+        <f t="array" aca="1" ref="O4" ca="1">_FV(L3,"Year incorporated",TRUE)</f>
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="5" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
         <v>117</v>
       </c>
@@ -1783,7 +2287,7 @@
         <v>3949547.3939999999</v>
       </c>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>117</v>
       </c>
@@ -1794,11 +2298,11 @@
         <v>39</v>
       </c>
       <c r="L6" s="1">
-        <f>L5*L4</f>
-        <v>1377404653.6575</v>
-      </c>
-    </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.25">
+        <f ca="1">L5*L4</f>
+        <v>1501301955.40728</v>
+      </c>
+    </row>
+    <row r="7" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>128</v>
       </c>
@@ -1810,7 +2314,7 @@
         <v>43524</v>
       </c>
     </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:15" x14ac:dyDescent="0.2">
       <c r="K8" t="s">
         <v>41</v>
       </c>
@@ -1819,51 +2323,51 @@
         <v>9342</v>
       </c>
     </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:15" x14ac:dyDescent="0.2">
       <c r="K9" t="s">
         <v>42</v>
       </c>
       <c r="L9" s="1">
-        <f>L6-L7+L8</f>
-        <v>1377370471.6575</v>
-      </c>
-    </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.25">
+        <f ca="1">L6-L7+L8</f>
+        <v>1501267773.40728</v>
+      </c>
+    </row>
+    <row r="10" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:15" x14ac:dyDescent="0.2">
       <c r="K15" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:15" x14ac:dyDescent="0.2">
       <c r="K16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>114</v>
       </c>
@@ -1871,7 +2375,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
         <v>115</v>
       </c>
@@ -1879,7 +2383,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
         <v>106</v>
       </c>
@@ -1887,32 +2391,32 @@
         <v>122</v>
       </c>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C23" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C24" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C26" t="s">
         <v>131</v>
       </c>
@@ -1920,37 +2424,37 @@
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C28" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C29" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C30" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C31" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C32" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C34" t="s">
         <v>112</v>
       </c>
@@ -1964,39 +2468,39 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3DD1473-2AA8-9C48-B00A-DBC01DC80D0B}">
   <dimension ref="B4:B11"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>133</v>
       </c>
@@ -2009,13 +2513,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68BB641C-A60E-1D48-998E-8C4C1E1253D6}">
   <dimension ref="A1:CU96"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
     <col min="3" max="41" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:99" x14ac:dyDescent="0.2">
       <c r="C1" s="15" t="s">
         <v>177</v>
       </c>
@@ -2212,7 +2716,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:99" x14ac:dyDescent="0.2">
       <c r="C2" s="13" t="s">
         <v>138</v>
       </c>
@@ -2502,7 +3006,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="3" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:99" x14ac:dyDescent="0.2">
       <c r="AP3" s="2"/>
       <c r="AQ3" s="2"/>
       <c r="AR3" s="2"/>
@@ -2530,7 +3034,7 @@
       <c r="BN3" s="2"/>
       <c r="BO3" s="2"/>
     </row>
-    <row r="4" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:99" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -2564,7 +3068,7 @@
       <c r="BN4" s="2"/>
       <c r="BO4" s="2"/>
     </row>
-    <row r="5" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:99" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>105</v>
       </c>
@@ -2595,7 +3099,7 @@
       <c r="BN5" s="2"/>
       <c r="BO5" s="2"/>
     </row>
-    <row r="6" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:99" x14ac:dyDescent="0.2">
       <c r="AP6" s="2"/>
       <c r="AQ6" s="2"/>
       <c r="AR6" s="2"/>
@@ -2623,7 +3127,7 @@
       <c r="BN6" s="2"/>
       <c r="BO6" s="2"/>
     </row>
-    <row r="7" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:99" x14ac:dyDescent="0.2">
       <c r="AP7" s="2"/>
       <c r="AQ7" s="2"/>
       <c r="AR7" s="2"/>
@@ -2651,7 +3155,7 @@
       <c r="BN7" s="2"/>
       <c r="BO7" s="2"/>
     </row>
-    <row r="8" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:99" x14ac:dyDescent="0.2">
       <c r="AP8" s="2"/>
       <c r="AQ8" s="2"/>
       <c r="AR8" s="2"/>
@@ -2679,7 +3183,7 @@
       <c r="BN8" s="2"/>
       <c r="BO8" s="2"/>
     </row>
-    <row r="9" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:99" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -2747,7 +3251,7 @@
       <c r="BN9" s="2"/>
       <c r="BO9" s="2"/>
     </row>
-    <row r="10" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
         <v>93</v>
       </c>
@@ -2786,7 +3290,7 @@
       <c r="BT10" s="11"/>
       <c r="BU10" s="11"/>
     </row>
-    <row r="11" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="s">
         <v>94</v>
       </c>
@@ -2825,7 +3329,7 @@
       <c r="BT11" s="11"/>
       <c r="BU11" s="11"/>
     </row>
-    <row r="12" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
         <v>95</v>
       </c>
@@ -2862,7 +3366,7 @@
       <c r="BQ12" s="1"/>
       <c r="BR12" s="1"/>
     </row>
-    <row r="13" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="AP13" s="9"/>
       <c r="AQ13" s="9"/>
       <c r="AR13" s="9"/>
@@ -2893,7 +3397,7 @@
       <c r="BQ13" s="1"/>
       <c r="BR13" s="1"/>
     </row>
-    <row r="14" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
         <v>96</v>
       </c>
@@ -2927,7 +3431,7 @@
       <c r="BQ14" s="1"/>
       <c r="BR14" s="1"/>
     </row>
-    <row r="15" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B15" s="7" t="s">
         <v>97</v>
       </c>
@@ -2961,7 +3465,7 @@
       <c r="BQ15" s="1"/>
       <c r="BR15" s="1"/>
     </row>
-    <row r="16" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:99" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="AP16" s="9"/>
       <c r="AQ16" s="9"/>
       <c r="AR16" s="9"/>
@@ -2992,7 +3496,7 @@
       <c r="BQ16" s="1"/>
       <c r="BR16" s="1"/>
     </row>
-    <row r="17" spans="2:67" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:67" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="AP17" s="9"/>
       <c r="AQ17" s="9"/>
       <c r="AR17" s="9"/>
@@ -3020,7 +3524,7 @@
       <c r="BN17" s="9"/>
       <c r="BO17" s="9"/>
     </row>
-    <row r="18" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -3088,7 +3592,7 @@
       <c r="BN18" s="2"/>
       <c r="BO18" s="2"/>
     </row>
-    <row r="19" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>45</v>
       </c>
@@ -3108,7 +3612,7 @@
         <v>20006</v>
       </c>
     </row>
-    <row r="20" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>49</v>
       </c>
@@ -3128,14 +3632,14 @@
         <v>16866</v>
       </c>
     </row>
-    <row r="22" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK22" s="1"/>
       <c r="BL22" s="1"/>
       <c r="BM22" s="1"/>
       <c r="BN22" s="1"/>
       <c r="BO22" s="1"/>
     </row>
-    <row r="23" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>47</v>
       </c>
@@ -3155,7 +3659,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="24" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>51</v>
       </c>
@@ -3175,14 +3679,14 @@
         <v>187</v>
       </c>
     </row>
-    <row r="26" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK26" s="1"/>
       <c r="BL26" s="1"/>
       <c r="BM26" s="1"/>
       <c r="BN26" s="1"/>
       <c r="BO26" s="1"/>
     </row>
-    <row r="27" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>46</v>
       </c>
@@ -3202,14 +3706,14 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK28" s="1"/>
       <c r="BL28" s="1"/>
       <c r="BM28" s="1"/>
       <c r="BN28" s="1"/>
       <c r="BO28" s="1"/>
     </row>
-    <row r="29" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>65</v>
       </c>
@@ -3234,7 +3738,7 @@
         <v>0.15695291412576229</v>
       </c>
     </row>
-    <row r="30" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>66</v>
       </c>
@@ -3259,14 +3763,14 @@
         <v>0.48626373626373631</v>
       </c>
     </row>
-    <row r="31" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK31" s="1"/>
       <c r="BL31" s="1"/>
       <c r="BM31" s="1"/>
       <c r="BN31" s="1"/>
       <c r="BO31" s="1"/>
     </row>
-    <row r="32" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>43</v>
       </c>
@@ -3291,21 +3795,21 @@
         <v>20516</v>
       </c>
     </row>
-    <row r="33" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK33" s="1"/>
       <c r="BL33" s="1"/>
       <c r="BM33" s="1"/>
       <c r="BN33" s="1"/>
       <c r="BO33" s="1"/>
     </row>
-    <row r="34" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK34" s="1"/>
       <c r="BL34" s="1"/>
       <c r="BM34" s="1"/>
       <c r="BN34" s="1"/>
       <c r="BO34" s="1"/>
     </row>
-    <row r="35" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>98</v>
       </c>
@@ -3325,7 +3829,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="37" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>44</v>
       </c>
@@ -3345,7 +3849,7 @@
         <v>3139</v>
       </c>
     </row>
-    <row r="38" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
         <v>52</v>
       </c>
@@ -3365,7 +3869,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="39" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
@@ -3407,7 +3911,7 @@
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
     </row>
-    <row r="40" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
         <v>48</v>
       </c>
@@ -3427,7 +3931,7 @@
         <v>4581</v>
       </c>
     </row>
-    <row r="41" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>53</v>
       </c>
@@ -3447,14 +3951,14 @@
         <v>3933</v>
       </c>
     </row>
-    <row r="42" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:67" x14ac:dyDescent="0.2">
       <c r="BK42" s="5"/>
       <c r="BL42" s="5"/>
       <c r="BM42" s="5"/>
       <c r="BN42" s="5"/>
       <c r="BO42" s="5"/>
     </row>
-    <row r="43" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>64</v>
       </c>
@@ -3479,7 +3983,7 @@
         <v>0.16879508676155197</v>
       </c>
     </row>
-    <row r="44" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>62</v>
       </c>
@@ -3504,7 +4008,7 @@
         <v>0.20388658808537752</v>
       </c>
     </row>
-    <row r="45" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>63</v>
       </c>
@@ -3529,7 +4033,7 @@
         <v>0.14145383104125742</v>
       </c>
     </row>
-    <row r="47" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B47" s="3" t="s">
         <v>0</v>
       </c>
@@ -3554,7 +4058,7 @@
         <v>28236</v>
       </c>
     </row>
-    <row r="48" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>54</v>
       </c>
@@ -3579,7 +4083,7 @@
         <v>23485</v>
       </c>
     </row>
-    <row r="49" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
         <v>61</v>
       </c>
@@ -3604,7 +4108,7 @@
         <v>4751</v>
       </c>
     </row>
-    <row r="50" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
         <v>55</v>
       </c>
@@ -3624,7 +4128,7 @@
         <v>2371</v>
       </c>
     </row>
-    <row r="51" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>56</v>
       </c>
@@ -3644,7 +4148,7 @@
         <v>1982</v>
       </c>
     </row>
-    <row r="52" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>57</v>
       </c>
@@ -3664,7 +4168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>58</v>
       </c>
@@ -3689,7 +4193,7 @@
         <v>4353</v>
       </c>
     </row>
-    <row r="54" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
         <v>60</v>
       </c>
@@ -3714,7 +4218,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="55" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>71</v>
       </c>
@@ -3739,7 +4243,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="56" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>72</v>
       </c>
@@ -3760,7 +4264,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="57" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>68</v>
       </c>
@@ -3780,7 +4284,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="58" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
         <v>70</v>
       </c>
@@ -3805,8 +4309,8 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="59" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="2:67" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:67" s="3" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="2:67" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B60" s="7" t="s">
         <v>69</v>
       </c>
@@ -3831,7 +4335,7 @@
         <v>0.15124153498871332</v>
       </c>
     </row>
-    <row r="62" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
         <v>50</v>
       </c>
@@ -3856,7 +4360,7 @@
         <v>0.16826037682391271</v>
       </c>
     </row>
-    <row r="63" spans="2:67" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:67" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>59</v>
       </c>
@@ -3881,7 +4385,7 @@
         <v>1.4095480946309675E-2</v>
       </c>
     </row>
-    <row r="68" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
         <v>73</v>
       </c>
@@ -3908,7 +4412,7 @@
       <c r="BT68" s="1"/>
       <c r="BU68" s="1"/>
     </row>
-    <row r="69" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
         <v>74</v>
       </c>
@@ -3934,7 +4438,7 @@
       <c r="BT69" s="1"/>
       <c r="BU69" s="1"/>
     </row>
-    <row r="70" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
         <v>75</v>
       </c>
@@ -3960,7 +4464,7 @@
       <c r="BT70" s="1"/>
       <c r="BU70" s="1"/>
     </row>
-    <row r="71" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
         <v>76</v>
       </c>
@@ -3986,7 +4490,7 @@
       <c r="BT71" s="1"/>
       <c r="BU71" s="1"/>
     </row>
-    <row r="72" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
         <v>77</v>
       </c>
@@ -4010,7 +4514,7 @@
       <c r="BT72" s="1"/>
       <c r="BU72" s="1"/>
     </row>
-    <row r="73" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
         <v>78</v>
       </c>
@@ -4034,7 +4538,7 @@
       <c r="BT73" s="1"/>
       <c r="BU73" s="1"/>
     </row>
-    <row r="74" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
         <v>79</v>
       </c>
@@ -4058,7 +4562,7 @@
       <c r="BT74" s="1"/>
       <c r="BU74" s="1"/>
     </row>
-    <row r="75" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>80</v>
       </c>
@@ -4082,7 +4586,7 @@
       <c r="BT75" s="1"/>
       <c r="BU75" s="1"/>
     </row>
-    <row r="76" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
         <v>81</v>
       </c>
@@ -4106,7 +4610,7 @@
       <c r="BT76" s="1"/>
       <c r="BU76" s="1"/>
     </row>
-    <row r="77" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
         <v>82</v>
       </c>
@@ -4130,7 +4634,7 @@
       <c r="BT77" s="1"/>
       <c r="BU77" s="1"/>
     </row>
-    <row r="78" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
         <v>67</v>
       </c>
@@ -4154,7 +4658,7 @@
       <c r="BT78" s="1"/>
       <c r="BU78" s="1"/>
     </row>
-    <row r="79" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
         <v>83</v>
       </c>
@@ -4185,7 +4689,7 @@
       <c r="BT79" s="1"/>
       <c r="BU79" s="1"/>
     </row>
-    <row r="80" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:73" x14ac:dyDescent="0.2">
       <c r="BK80" s="1"/>
       <c r="BL80" s="1"/>
       <c r="BM80" s="1"/>
@@ -4198,7 +4702,7 @@
       <c r="BT80" s="1"/>
       <c r="BU80" s="1"/>
     </row>
-    <row r="81" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
         <v>84</v>
       </c>
@@ -4222,7 +4726,7 @@
       <c r="BT81" s="1"/>
       <c r="BU81" s="1"/>
     </row>
-    <row r="82" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
         <v>85</v>
       </c>
@@ -4246,7 +4750,7 @@
       <c r="BT82" s="1"/>
       <c r="BU82" s="1"/>
     </row>
-    <row r="83" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
         <v>88</v>
       </c>
@@ -4270,7 +4774,7 @@
       <c r="BT83" s="1"/>
       <c r="BU83" s="1"/>
     </row>
-    <row r="84" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
         <v>86</v>
       </c>
@@ -4294,7 +4798,7 @@
       <c r="BT84" s="1"/>
       <c r="BU84" s="1"/>
     </row>
-    <row r="85" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
         <v>87</v>
       </c>
@@ -4318,7 +4822,7 @@
       <c r="BT85" s="1"/>
       <c r="BU85" s="1"/>
     </row>
-    <row r="86" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
         <v>89</v>
       </c>
@@ -4342,7 +4846,7 @@
       <c r="BT86" s="1"/>
       <c r="BU86" s="1"/>
     </row>
-    <row r="87" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
         <v>90</v>
       </c>
@@ -4366,7 +4870,7 @@
       <c r="BT87" s="1"/>
       <c r="BU87" s="1"/>
     </row>
-    <row r="88" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
         <v>91</v>
       </c>
@@ -4397,7 +4901,7 @@
       <c r="BT88" s="1"/>
       <c r="BU88" s="1"/>
     </row>
-    <row r="89" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:73" x14ac:dyDescent="0.2">
       <c r="BK89" s="1"/>
       <c r="BL89" s="1"/>
       <c r="BM89" s="1"/>
@@ -4410,7 +4914,7 @@
       <c r="BT89" s="1"/>
       <c r="BU89" s="1"/>
     </row>
-    <row r="90" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
         <v>126</v>
       </c>
@@ -4430,8 +4934,8 @@
       <c r="BT90" s="1"/>
       <c r="BU90" s="1"/>
     </row>
-    <row r="91" spans="2:73" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:73" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="92" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B92" t="s">
         <v>92</v>
       </c>
@@ -4462,7 +4966,7 @@
       <c r="BT92" s="1"/>
       <c r="BU92" s="1"/>
     </row>
-    <row r="93" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
         <v>124</v>
       </c>
@@ -4476,7 +4980,7 @@
         <v>3949</v>
       </c>
     </row>
-    <row r="94" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:73" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
         <v>125</v>
       </c>
@@ -4487,7 +4991,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="96" spans="2:73" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:73" x14ac:dyDescent="0.2">
       <c r="BM96" s="1"/>
     </row>
   </sheetData>

</xml_diff>